<commit_message>
correcciones de estilos y nuevos mensajes
</commit_message>
<xml_diff>
--- a/public/INVITADOS MATRIMONIO CARLOS Y VALENTINA.xlsx
+++ b/public/INVITADOS MATRIMONIO CARLOS Y VALENTINA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nicolth\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\Codigo\CarVal\boda-angular\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E7DE369-C682-4B2B-8772-C719F8FA095B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F8826B-8482-4A39-AA02-5AC38A201664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{6575D534-036F-4B88-9277-9285B9674B78}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6575D534-036F-4B88-9277-9285B9674B78}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>PARA</t>
   </si>
@@ -47,12 +47,6 @@
     <t>N° DE CUPOS</t>
   </si>
   <si>
-    <t>4 PERSONAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 PERSONAS </t>
-  </si>
-  <si>
     <t>FLIA GOMEZ PERDOMO</t>
   </si>
   <si>
@@ -83,12 +77,6 @@
     <t>FLIA MONTEALEGRE AGUILAR</t>
   </si>
   <si>
-    <t>3 PERSONAS</t>
-  </si>
-  <si>
-    <t>5 PERSONAS</t>
-  </si>
-  <si>
     <t>CESAR ALBERTO AGUILAR RODRIGUEZ</t>
   </si>
   <si>
@@ -104,9 +92,6 @@
     <t xml:space="preserve">SANDRA ESPINOZA </t>
   </si>
   <si>
-    <t>1 PERSONA</t>
-  </si>
-  <si>
     <t xml:space="preserve">JIMENA LOSADA  Y ESPOSA </t>
   </si>
   <si>
@@ -117,6 +102,12 @@
   </si>
   <si>
     <t xml:space="preserve">ANDRES FELIPE BOLIVAR Y ESPOSA </t>
+  </si>
+  <si>
+    <t>SRA. MARÍA FERNANDA GOMEZ PERDOMO</t>
+  </si>
+  <si>
+    <t>BRAYAN ROJAS</t>
   </si>
 </sst>
 </file>
@@ -488,14 +479,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34CAA6C4-DD28-48D9-A14D-637B0067F923}">
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.54296875" customWidth="1"/>
-    <col min="2" max="2" width="22.08984375" customWidth="1"/>
+    <col min="1" max="1" width="49.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -503,169 +494,173 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
         <v>5</v>
       </c>
-      <c r="B4" t="str">
-        <f>B3</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="str">
-        <f>B4</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="str">
-        <f>B5</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="str">
-        <f>B6</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" t="str">
-        <f>B7</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <f>B18</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="str">
-        <f>B9</f>
-        <v>1 PERSONA</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" t="str">
-        <f>B9</f>
-        <v>1 PERSONA</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" t="str">
-        <f>B9</f>
-        <v>1 PERSONA</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" t="str">
-        <f>B14</f>
-        <v>1 PERSONA</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>22</v>
       </c>
-      <c r="B16" t="str">
-        <f>B18</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" t="str">
-        <f>B13</f>
-        <v>1 PERSONA</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" t="str">
-        <f>B7</f>
-        <v xml:space="preserve">2 PERSONAS </v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" t="str">
-        <f>B17</f>
-        <v>1 PERSONA</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" t="s">
-        <v>3</v>
+      <c r="B22">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>